<commit_message>
tabtools: SSC pre-release polish (1.0.0, 2026-10-15)
Unified Exported line with true sheet dimensions; no -0.00 at any number
formatting site; survtab N with separators; wrapped small-cell notes;
footnote paragraph splitting in hrcomptab/stacktab; help example fixes;
corrtab leftovers removed; README command count.
</commit_message>
<xml_diff>
--- a/tabtools/demo/demo_effecttab.xlsx
+++ b/tabtools/demo/demo_effecttab.xlsx
@@ -43,7 +43,7 @@
     <t>95% CI</t>
   </si>
   <si>
-    <t>(-0.00, 0.05)</t>
+    <t>(0.00, 0.05)</t>
   </si>
   <si>
     <t>(0.33, 0.36)</t>
@@ -124,7 +124,7 @@
     <t>(-0.01, 0.03)</t>
   </si>
   <si>
-    <t>(-0.00, 0.00)</t>
+    <t>(0.00, 0.00)</t>
   </si>
   <si>
     <t>(-0.01, 0.02)</t>

</xml_diff>